<commit_message>
Publish settlements from settlement-cycle PR #117: feat(grove): address Grove findings — Maple syrupUSDC, Agora incentives, daily Debt xlsx tab
Source: https://github.com/soterlabs/settlement-cycle/pull/117
</commit_message>
<xml_diff>
--- a/reports/grove/2026-01/grove_settlement_january_2026.xlsx
+++ b/reports/grove/2026-01/grove_settlement_january_2026.xlsx
@@ -11,8 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sky Revenue" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sky Direct" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Off-protocol holdings" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SDE daily" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Off-protocol holdings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SDE daily" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -76,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -89,6 +90,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -652,7 +654,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-06-05T11:08:01+00:00</t>
+          <t>2026-06-08T08:17:40+00:00</t>
         </is>
       </c>
     </row>
@@ -679,7 +681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S30"/>
+  <dimension ref="A1:S32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2058,12 +2060,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>E11</t>
+          <t>E37</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Curve AUSD/USDC stableswap LP</t>
+          <t>Maple syrupUSDC (ERC-4626)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2073,7 +2075,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
@@ -2123,12 +2125,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>E13</t>
+          <t>E11</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>RLUSD raw (ALM idle)</t>
+          <t>Curve AUSD/USDC stableswap LP</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2138,7 +2140,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E22" s="5" t="n">
@@ -2188,12 +2190,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>E16</t>
+          <t>E13</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DAI raw (ALM idle)</t>
+          <t>RLUSD raw (ALM idle)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2253,12 +2255,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>E17</t>
+          <t>E16</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>USDS raw / POL (ALM idle — already netted out of utilized)</t>
+          <t>DAI raw (ALM idle)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2296,7 +2298,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N24" s="5" t="n">
         <v>0</v>
@@ -2313,21 +2315,17 @@
       <c r="R24" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>CoF excluded (already deducted from utilized)</t>
-        </is>
-      </c>
+      <c r="S24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>E18</t>
+          <t>E17</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>sUSDS raw / POL (ALM idle — Cat B 4626)</t>
+          <t>USDS raw / POL (ALM idle — already netted out of utilized)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2337,7 +2335,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E25" s="5" t="n">
@@ -2365,7 +2363,7 @@
         <v>0</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N25" s="5" t="n">
         <v>0</v>
@@ -2382,22 +2380,26 @@
       <c r="R25" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="S25" t="inlineStr"/>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>CoF excluded (already deducted from utilized)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>E23</t>
+          <t>E18</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Steakhouse Prime Instant (Base, Morpho V2)</t>
+          <t>sUSDS raw / POL (ALM idle — Cat B 4626)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2452,17 +2454,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>E24</t>
+          <t>E23</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Steakhouse High Yield PYUSD (Morpho 4626)</t>
+          <t>Steakhouse Prime Instant (Base, Morpho V2)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2517,12 +2519,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>E26</t>
+          <t>E24</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PYUSD raw (ALM idle)</t>
+          <t>Steakhouse High Yield PYUSD (Morpho 4626)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2532,7 +2534,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E28" s="5" t="n">
@@ -2582,17 +2584,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>E27</t>
+          <t>E26</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>USDC raw on Base (ALM idle)</t>
+          <t>PYUSD raw (ALM idle)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2647,59 +2649,189 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>E27</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>USDC raw on Base (ALM idle)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>E38</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Agora AUSD incentives (cash distribution to Grove Eth ALM)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ethereum</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>PSM_CURVE_DEDUCT</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>PSM3 USDS + PSM3 USDC (SDE) + Curve idle USDS — BR deduction (unattributed)</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S30" t="inlineStr">
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" t="inlineStr">
         <is>
           <t>BR deduction from PSM3 USDS leg + PSM3 USDC leg (SDE, ≈$0 yield) + Curve idle USDS — not tracked per-venue; residual = sky_rev_br_reduction − Σ(known venue deduction_avg × effective_br_rate × n_days)</t>
         </is>
@@ -3145,6 +3277,1671 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Daily ilk debt + Sky charge breakdown</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>cum_debt = Σ on-chain Vat dart from frob (0x76088703) + grab (0x7bab3f40). utilized = cum_debt − Σ deductions. base_apy = (1+SSR)(1+0.003)−1 (multiplicative). sub_apy applies on the first cap_usd of utilized when the subsidy is active; excess pays base_apy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>cum_debt</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>− ALM idle</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>− PSM USDS</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>− SDE NAV</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>− Curve idle</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>− Lending idle</t>
+        </is>
+      </c>
+      <c r="H5" s="2">
+        <f> utilized</f>
+        <v/>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>SSR APY</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>base APY</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>T (months)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>ref_rate APY</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>sub APY</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>daily Sky charge</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>daily Sky charge (gross on cum_debt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1984828055.219324</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>762824824.7566538</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>1222003230.46267</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M6" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>124430.2757766502</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>212664.3707622077</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-01-02</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>1985828055.219324</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>762860738.2166537</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>1222967317.00267</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N7" s="3" t="n">
+        <v>124541.7893254808</v>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>212780.0383337419</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1985828055.219324</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>762860738.2166537</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>1222967317.00267</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M8" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>124541.7893254808</v>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>212780.0383337419</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-01-04</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1985828055.219324</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>762900103.7688839</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>1222927951.45044</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N9" s="3" t="n">
+        <v>124537.2360076522</v>
+      </c>
+      <c r="O9" s="3" t="n">
+        <v>212780.0383337419</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>1995828055.219324</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>763022687.8884877</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>1232805367.330836</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M10" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>125679.7327155704</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>213936.7140490833</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-01-06</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>2012328055.219324</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>763063046.3086326</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>1249265008.910691</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N11" s="3" t="n">
+        <v>127583.5794854346</v>
+      </c>
+      <c r="O11" s="3" t="n">
+        <v>215845.2289793966</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>2006577041.234456</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>803105106.0675159</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>1203471935.16694</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M12" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N12" s="3" t="n">
+        <v>122286.8058524111</v>
+      </c>
+      <c r="O12" s="3" t="n">
+        <v>215180.023157908</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-01-08</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>2026577041.234456</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>803143978.3027297</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>1223433062.931726</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M13" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N13" s="3" t="n">
+        <v>124595.6610260466</v>
+      </c>
+      <c r="O13" s="3" t="n">
+        <v>217493.3745885908</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-01-09</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>1926524960.710924</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>823185735.0412451</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>1103339225.669679</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M14" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N14" s="3" t="n">
+        <v>110704.6985137294</v>
+      </c>
+      <c r="O14" s="3" t="n">
+        <v>205920.5934074957</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>1926524960.710924</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>823185735.0412451</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>1103339225.669679</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N15" s="3" t="n">
+        <v>110704.6985137294</v>
+      </c>
+      <c r="O15" s="3" t="n">
+        <v>205920.5934074957</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-01-11</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>1926524960.710924</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>823185735.0412451</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>1103339225.669679</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J16" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M16" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N16" s="3" t="n">
+        <v>110704.6985137294</v>
+      </c>
+      <c r="O16" s="3" t="n">
+        <v>205920.5934074957</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>1956524960.710924</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>843317637.3667084</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>1113207323.344216</v>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J17" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M17" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N17" s="3" t="n">
+        <v>111846.1174074048</v>
+      </c>
+      <c r="O17" s="3" t="n">
+        <v>209390.6205535199</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>1946290696.105259</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>903358721.0850873</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>1042931975.020172</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M18" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N18" s="3" t="n">
+        <v>103717.5385280469</v>
+      </c>
+      <c r="O18" s="3" t="n">
+        <v>208206.8480201448</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>1971790696.105259</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>903399116.9614611</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>1068391579.143798</v>
+      </c>
+      <c r="I19" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M19" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N19" s="3" t="n">
+        <v>106662.3891092473</v>
+      </c>
+      <c r="O19" s="3" t="n">
+        <v>211156.3710942654</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>1961776234.45376</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>943446845.432757</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>1018329389.021003</v>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J20" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M20" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N20" s="3" t="n">
+        <v>100871.8171520632</v>
+      </c>
+      <c r="O20" s="3" t="n">
+        <v>209998.0226348147</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>1961776234.45376</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>943500490.6691302</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>1018275743.78463</v>
+      </c>
+      <c r="I21" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M21" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N21" s="3" t="n">
+        <v>100865.6121378476</v>
+      </c>
+      <c r="O21" s="3" t="n">
+        <v>209998.0226348147</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1961776234.45376</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>943500490.6691302</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>1018275743.78463</v>
+      </c>
+      <c r="I22" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J22" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M22" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N22" s="3" t="n">
+        <v>100865.6121378476</v>
+      </c>
+      <c r="O22" s="3" t="n">
+        <v>209998.0226348147</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>1961776234.45376</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>943500490.6691302</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>1018275743.78463</v>
+      </c>
+      <c r="I23" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J23" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M23" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N23" s="3" t="n">
+        <v>100865.6121378476</v>
+      </c>
+      <c r="O23" s="3" t="n">
+        <v>209998.0226348147</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>1962777234.45376</v>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>943500490.6691302</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>1019276743.78463</v>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M24" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N24" s="3" t="n">
+        <v>100981.3953769532</v>
+      </c>
+      <c r="O24" s="3" t="n">
+        <v>210113.8058739204</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>1933909642.799006</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>963737271.2934443</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>970172371.5055617</v>
+      </c>
+      <c r="I25" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J25" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M25" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N25" s="3" t="n">
+        <v>95806.17217862917</v>
+      </c>
+      <c r="O25" s="3" t="n">
+        <v>206774.7616511758</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>1934309642.799006</v>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>983792436.63439</v>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>950517206.164616</v>
+      </c>
+      <c r="I26" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J26" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M26" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N26" s="3" t="n">
+        <v>93865.19116313005</v>
+      </c>
+      <c r="O26" s="3" t="n">
+        <v>206821.0286797895</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1972909642.799006</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>983848621.2736028</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>989061021.5254031</v>
+      </c>
+      <c r="I27" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J27" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M27" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N27" s="3" t="n">
+        <v>97671.45850214559</v>
+      </c>
+      <c r="O27" s="3" t="n">
+        <v>211285.7969410072</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1972909642.799006</v>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>983907696.0662968</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>989001946.7327092</v>
+      </c>
+      <c r="I28" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J28" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M28" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N28" s="3" t="n">
+        <v>97665.62476586687</v>
+      </c>
+      <c r="O28" s="3" t="n">
+        <v>211285.7969410072</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1974009642.799006</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>1003909435.032003</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>970100207.7670031</v>
+      </c>
+      <c r="I29" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J29" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M29" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N29" s="3" t="n">
+        <v>95799.04588667894</v>
+      </c>
+      <c r="O29" s="3" t="n">
+        <v>211413.0312696948</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>1974009642.799006</v>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>1003909435.032003</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>970100207.7670031</v>
+      </c>
+      <c r="I30" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J30" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M30" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N30" s="3" t="n">
+        <v>95799.04588667894</v>
+      </c>
+      <c r="O30" s="3" t="n">
+        <v>211413.0312696948</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>2007509642.799006</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>1004098132.792144</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>1003411510.006862</v>
+      </c>
+      <c r="I31" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J31" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M31" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N31" s="3" t="n">
+        <v>99146.30231405739</v>
+      </c>
+      <c r="O31" s="3" t="n">
+        <v>215287.8949160884</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>2007509642.799006</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>1024159461.833279</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>983350180.9657269</v>
+      </c>
+      <c r="I32" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J32" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M32" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N32" s="3" t="n">
+        <v>97107.50328138829</v>
+      </c>
+      <c r="O32" s="3" t="n">
+        <v>215287.8949160884</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>2027509642.799006</v>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>1024225089.412934</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>1003284553.386072</v>
+      </c>
+      <c r="I33" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J33" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M33" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N33" s="3" t="n">
+        <v>99131.61755004049</v>
+      </c>
+      <c r="O33" s="3" t="n">
+        <v>217601.2463467712</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>2049561642.799006</v>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>1044281848.307186</v>
+      </c>
+      <c r="F34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="5" t="n">
+        <v>1005279794.49182</v>
+      </c>
+      <c r="I34" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J34" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M34" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N34" s="3" t="n">
+        <v>99362.40224336745</v>
+      </c>
+      <c r="O34" s="3" t="n">
+        <v>220151.9476342421</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>2049561642.799006</v>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>1064349366.450599</v>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>985212276.3484071</v>
+      </c>
+      <c r="I35" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J35" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M35" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N35" s="3" t="n">
+        <v>97291.38836829222</v>
+      </c>
+      <c r="O35" s="3" t="n">
+        <v>220151.9476342421</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>2049561642.799006</v>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="5" t="n">
+        <v>1064349366.450599</v>
+      </c>
+      <c r="F36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="5" t="n">
+        <v>985212276.3484071</v>
+      </c>
+      <c r="I36" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J36" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M36" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N36" s="3" t="n">
+        <v>97291.38836829222</v>
+      </c>
+      <c r="O36" s="3" t="n">
+        <v>220151.9476342421</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Σ daily charges</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" s="10" t="n">
+        <v>3322924.199551741</v>
+      </c>
+      <c r="O38" s="10" t="n">
+        <v>6577707.668676052</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3438,7 +5235,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>